<commit_message>
docs(coverage): calibrate CVE-2026-115560 workbook transitions and scanner claims
- Demarcate 1 C-binary transition (PHP 8.1 on php81-mitigation) from 8 SAPI runtime hardening transitions in Summary and Verified Transitions sheets
- Accurately label container matrix results as 'RUNTIME HARDENED' for SAPI drop-ins and 'MITIGATED (403/Off)' for PHP 8.1
- Scope Akatsuki Lab attack sweep to probed target php81-mitigation over labbr0
- Explicitly add Status column to Oracle Finding sheet tagging delimiter key probe as 'INCONCLUSIVE' and others as 'PASS'
- Re-generate docs/test-report/cve-2026-115560-coverage-metrix.xlsx with calibrated data and zero unverified assertions
</commit_message>
<xml_diff>
--- a/docs/test-report/cve-2026-115560-coverage-matrix-2026-10-24.xlsx
+++ b/docs/test-report/cve-2026-115560-coverage-matrix-2026-10-24.xlsx
@@ -18,12 +18,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Artifacts" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$12:$C$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$12:$C$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Container Matrix'!$A$5:$G$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Verified Transitions'!$A$5:$G$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Range Coverage'!$A$5:$F$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Scope'!$A$5:$D$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Oracle Finding'!$A$5:$D$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Oracle Finding'!$A$5:$E$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Docker Suite'!$A$5:$E$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Patch Inventory'!$A$5:$D$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Artifacts'!$A$5:$D$17</definedName>
@@ -243,7 +243,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -287,6 +287,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -655,7 +658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
@@ -706,12 +709,12 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED TRANSITIONS</t>
+          <t>C-BINARY VERIFIED</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>CONTAINER HARNESS</t>
+          <t>RUNTIME SAPI PASS</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -734,10 +737,10 @@
         <v>1</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G6" s="10" t="n">
         <v>9</v>
@@ -751,7 +754,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>C-BINARY VERIFIED</t>
+          <t>C-BINARY FIX</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -807,7 +810,7 @@
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>Akatsuki Lab sweep — all targets</t>
+          <t>Akatsuki Lab attack sweep</t>
         </is>
       </c>
       <c r="B13" s="13" t="inlineStr">
@@ -817,7 +820,7 @@
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>9/9 sampled targets verified, edge drops HTTP 403, 0 failures</t>
+          <t>Probed php81-mitigation over labbr0; edge drops HTTP 403, testploit MITIGATED</t>
         </is>
       </c>
     </row>
@@ -841,7 +844,7 @@
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>Fix-mode coverage</t>
+          <t>Fix-mode distribution</t>
         </is>
       </c>
       <c r="B15" s="13" t="inlineStr">
@@ -851,14 +854,14 @@
       </c>
       <c r="C15" s="14" t="inlineStr">
         <is>
-          <t>9 of 9 sampled targets verified: 1 C-binary (PHP 8.1), 8 runtime SAPI drop-in</t>
+          <t>1 target C-binary rebuilt (PHP 8.1); 8 targets hardened via runtime SAPI drop-in</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>Vulnerable → mitigated transitions</t>
+          <t>Runtime SAPI transitions</t>
         </is>
       </c>
       <c r="B16" s="13" t="inlineStr">
@@ -868,14 +871,14 @@
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>9 targets: PHP 5.5 through 8.4 across Ubuntu, Debian, Alpine — each scanned before and after</t>
+          <t>9 sampled targets: session.upload_progress.enabled transitioned from On to Off</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>PHP version changed by the fix</t>
+          <t>C-Binary engine transition</t>
         </is>
       </c>
       <c r="B17" s="13" t="inlineStr">
@@ -885,14 +888,14 @@
       </c>
       <c r="C17" s="14" t="inlineStr">
         <is>
-          <t>Drop-in &amp; backport only; version string identical before and after on every target</t>
+          <t>1 target (PHP 8.1): stock binary transitioned to key-sanitized C-binary</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>Served binary matches built binary</t>
+          <t>PHP version changed by the fix</t>
         </is>
       </c>
       <c r="B18" s="13" t="inlineStr">
@@ -902,14 +905,14 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>SHA-256 of the running FPM binary on php81-mitigation equals the freshly built one</t>
+          <t>Drop-in &amp; backport only; version string identical before and after on every target</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>Scope</t>
+          <t>Served binary matches built binary</t>
         </is>
       </c>
       <c r="B19" s="13" t="inlineStr">
@@ -919,31 +922,31 @@
       </c>
       <c r="C19" s="14" t="inlineStr">
         <is>
-          <t>Sampled environments across Ubuntu 14.04-24.04, Debian 12, Alpine 3.21, and PHP 8.4-FPM</t>
+          <t>SHA-256 of the running FPM binary on php81-mitigation equals the freshly built one</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>Cross-OS Docker suite</t>
+          <t>Sampled scope coverage</t>
         </is>
       </c>
       <c r="B20" s="13" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>debian12 (PHP 8.2), alpine (PHP 8.3), php8.4-fpm (PHP 8.4) — all PASS, zero failures</t>
+          <t>Sampled environments across Ubuntu 14.04-24.04, Debian 12, Alpine 3.21, and PHP 8.4-FPM</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>Perimeter filter trip</t>
+          <t>Cross-OS Docker suite</t>
         </is>
       </c>
       <c r="B21" s="13" t="inlineStr">
@@ -953,29 +956,46 @@
       </c>
       <c r="C21" s="14" t="inlineStr">
         <is>
-          <t>Nginx edge filter drops PHP_SESSION_UPLOAD_PROGRESS marker with HTTP 403 Forbidden</t>
+          <t>debian12 (PHP 8.2), alpine (PHP 8.3), php8.4-fpm (PHP 8.4) — all PASS, zero failures</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="15" t="inlineStr">
         <is>
+          <t>Perimeter filter trip</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C22" s="16" t="inlineStr">
+        <is>
+          <t>Nginx edge filter drops PHP_SESSION_UPLOAD_PROGRESS marker with HTTP 403 Forbidden</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
           <t>Multi-CVE coexistence</t>
         </is>
       </c>
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="C22" s="16" t="inlineStr">
+      <c r="C23" s="14" t="inlineStr">
         <is>
           <t>Sequential patch with CVE-109618-109619 cleanly applied (--fuzz=0, exit 0)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A12:C22"/>
+  <autoFilter ref="A12:C23"/>
   <mergeCells count="2">
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A2:H2"/>
@@ -997,7 +1017,7 @@
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
     <col width="62" customWidth="1" min="7" max="7"/>
   </cols>
@@ -1045,7 +1065,7 @@
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>Scanner verdict</t>
+          <t>Verification Result</t>
         </is>
       </c>
       <c r="F5" s="11" t="inlineStr">
@@ -1082,7 +1102,7 @@
       </c>
       <c r="E6" s="12" t="inlineStr">
         <is>
-          <t>MITIGATED</t>
+          <t>RUNTIME HARDENED</t>
         </is>
       </c>
       <c r="F6" s="13" t="inlineStr">
@@ -1092,7 +1112,7 @@
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>Drop-in installed; TCP 9010; SAPI Off; rollback clean</t>
+          <t>Drop-in verified; TCP 9010; SAPI Off; rollback clean</t>
         </is>
       </c>
     </row>
@@ -1119,7 +1139,7 @@
       </c>
       <c r="E7" s="15" t="inlineStr">
         <is>
-          <t>MITIGATED</t>
+          <t>RUNTIME HARDENED</t>
         </is>
       </c>
       <c r="F7" s="13" t="inlineStr">
@@ -1129,7 +1149,7 @@
       </c>
       <c r="G7" s="16" t="inlineStr">
         <is>
-          <t>Drop-in installed; UNIX socket; SAPI Off; rollback clean</t>
+          <t>Drop-in verified; UNIX socket; SAPI Off; rollback clean</t>
         </is>
       </c>
     </row>
@@ -1156,7 +1176,7 @@
       </c>
       <c r="E8" s="12" t="inlineStr">
         <is>
-          <t>MITIGATED</t>
+          <t>RUNTIME HARDENED</t>
         </is>
       </c>
       <c r="F8" s="13" t="inlineStr">
@@ -1166,7 +1186,7 @@
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
-          <t>Drop-in installed; TCP 9005; SAPI Off; rollback clean</t>
+          <t>Drop-in verified; TCP 9005; SAPI Off; rollback clean</t>
         </is>
       </c>
     </row>
@@ -1193,7 +1213,7 @@
       </c>
       <c r="E9" s="15" t="inlineStr">
         <is>
-          <t>MITIGATED</t>
+          <t>RUNTIME HARDENED</t>
         </is>
       </c>
       <c r="F9" s="13" t="inlineStr">
@@ -1203,7 +1223,7 @@
       </c>
       <c r="G9" s="16" t="inlineStr">
         <is>
-          <t>Drop-in installed; UNIX socket; SIGUSR2 reload; SAPI Off; rollback clean</t>
+          <t>Drop-in verified; UNIX socket; SIGUSR2 reload; SAPI Off; rollback clean</t>
         </is>
       </c>
     </row>
@@ -1230,7 +1250,7 @@
       </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
-          <t>MITIGATED</t>
+          <t>RUNTIME HARDENED</t>
         </is>
       </c>
       <c r="F10" s="13" t="inlineStr">
@@ -1240,7 +1260,7 @@
       </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
-          <t>Drop-in installed; UNIX socket; SIGUSR2 reload; SAPI Off; rollback clean</t>
+          <t>Drop-in verified; UNIX socket; SIGUSR2 reload; SAPI Off; rollback clean</t>
         </is>
       </c>
     </row>
@@ -1267,7 +1287,7 @@
       </c>
       <c r="E11" s="15" t="inlineStr">
         <is>
-          <t>MITIGATED</t>
+          <t>MITIGATED (403/Off)</t>
         </is>
       </c>
       <c r="F11" s="13" t="inlineStr">
@@ -1304,7 +1324,7 @@
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>MITIGATED</t>
+          <t>RUNTIME HARDENED</t>
         </is>
       </c>
       <c r="F12" s="13" t="inlineStr">
@@ -1341,7 +1361,7 @@
       </c>
       <c r="E13" s="15" t="inlineStr">
         <is>
-          <t>MITIGATED</t>
+          <t>RUNTIME HARDENED</t>
         </is>
       </c>
       <c r="F13" s="13" t="inlineStr">
@@ -1378,7 +1398,7 @@
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>MITIGATED</t>
+          <t>RUNTIME HARDENED</t>
         </is>
       </c>
       <c r="F14" s="13" t="inlineStr">
@@ -1413,11 +1433,11 @@
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="59" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1436,7 +1456,7 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Scanned VULNERABLE before, MITIGATED after · configuration &amp; binary verified</t>
+          <t>State transitions before and after mitigation deployment</t>
         </is>
       </c>
     </row>
@@ -1453,22 +1473,22 @@
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
+          <t>Verification Scope</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
           <t>Before</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
+      <c r="E5" s="11" t="inlineStr">
         <is>
           <t>After</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
-        <is>
-          <t>Version unchanged</t>
-        </is>
-      </c>
       <c r="F5" s="11" t="inlineStr">
         <is>
-          <t>Binary / Drop-in Reference</t>
+          <t>Fix Mode</t>
         </is>
       </c>
       <c r="G5" s="11" t="inlineStr">
@@ -1490,27 +1510,27 @@
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
-          <t>VULNERABLE (200)</t>
+          <t>Runtime Configuration</t>
         </is>
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
-          <t>MITIGATED (403/Off)</t>
+          <t>UNHARDENED (SAPI On)</t>
         </is>
       </c>
       <c r="E6" s="12" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>HARDENED (SAPI Off)</t>
         </is>
       </c>
       <c r="F6" s="12" t="inlineStr">
         <is>
-          <t>cve-115560-ini-dropin</t>
+          <t>SAPI INI Drop-in</t>
         </is>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>Marker allowed before -&gt; blocked after; SAPI Off</t>
+          <t>99-cve-2026-115560-hardening.ini · SAPI verified Off</t>
         </is>
       </c>
     </row>
@@ -1527,27 +1547,27 @@
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>VULNERABLE (200)</t>
+          <t>Runtime Configuration</t>
         </is>
       </c>
       <c r="D7" s="15" t="inlineStr">
         <is>
-          <t>MITIGATED (403/Off)</t>
+          <t>UNHARDENED (SAPI On)</t>
         </is>
       </c>
       <c r="E7" s="15" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>HARDENED (SAPI Off)</t>
         </is>
       </c>
       <c r="F7" s="15" t="inlineStr">
         <is>
-          <t>cve-115560-ini-dropin</t>
+          <t>SAPI INI Drop-in</t>
         </is>
       </c>
       <c r="G7" s="16" t="inlineStr">
         <is>
-          <t>Marker allowed before -&gt; blocked after; SAPI Off</t>
+          <t>99-cve-2026-115560-hardening.ini · SAPI verified Off</t>
         </is>
       </c>
     </row>
@@ -1564,27 +1584,27 @@
       </c>
       <c r="C8" s="12" t="inlineStr">
         <is>
-          <t>VULNERABLE (200)</t>
+          <t>Runtime Configuration</t>
         </is>
       </c>
       <c r="D8" s="12" t="inlineStr">
         <is>
-          <t>MITIGATED (403/Off)</t>
+          <t>UNHARDENED (SAPI On)</t>
         </is>
       </c>
       <c r="E8" s="12" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>HARDENED (SAPI Off)</t>
         </is>
       </c>
       <c r="F8" s="12" t="inlineStr">
         <is>
-          <t>cve-115560-ini-dropin</t>
+          <t>SAPI INI Drop-in</t>
         </is>
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
-          <t>Marker allowed before -&gt; blocked after; SAPI Off</t>
+          <t>99-cve-2026-115560-hardening.ini · SAPI verified Off</t>
         </is>
       </c>
     </row>
@@ -1601,27 +1621,27 @@
       </c>
       <c r="C9" s="15" t="inlineStr">
         <is>
-          <t>VULNERABLE (200)</t>
+          <t>Runtime Configuration</t>
         </is>
       </c>
       <c r="D9" s="15" t="inlineStr">
         <is>
-          <t>MITIGATED (403/Off)</t>
+          <t>UNHARDENED (SAPI On)</t>
         </is>
       </c>
       <c r="E9" s="15" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>HARDENED (SAPI Off)</t>
         </is>
       </c>
       <c r="F9" s="15" t="inlineStr">
         <is>
-          <t>cve-115560-ini-dropin</t>
+          <t>SAPI INI Drop-in</t>
         </is>
       </c>
       <c r="G9" s="16" t="inlineStr">
         <is>
-          <t>SIGUSR2 reloaded; SAPI Off; rollback verified</t>
+          <t>SIGUSR2 non-blocking reload · SAPI verified Off</t>
         </is>
       </c>
     </row>
@@ -1638,27 +1658,27 @@
       </c>
       <c r="C10" s="12" t="inlineStr">
         <is>
-          <t>VULNERABLE (200)</t>
+          <t>Runtime Configuration</t>
         </is>
       </c>
       <c r="D10" s="12" t="inlineStr">
         <is>
-          <t>MITIGATED (403/Off)</t>
+          <t>UNHARDENED (SAPI On)</t>
         </is>
       </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>HARDENED (SAPI Off)</t>
         </is>
       </c>
       <c r="F10" s="12" t="inlineStr">
         <is>
-          <t>cve-115560-ini-dropin</t>
+          <t>SAPI INI Drop-in</t>
         </is>
       </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
-          <t>SIGUSR2 reloaded; SAPI Off; rollback verified</t>
+          <t>SIGUSR2 non-blocking reload · SAPI verified Off</t>
         </is>
       </c>
     </row>
@@ -1675,27 +1695,27 @@
       </c>
       <c r="C11" s="15" t="inlineStr">
         <is>
-          <t>VULNERABLE (200)</t>
+          <t>C-Binary Rebuild &amp; Probe</t>
         </is>
       </c>
       <c r="D11" s="15" t="inlineStr">
         <is>
-          <t>MITIGATED (403/Off)</t>
+          <t>VULNERABLE (200 / On)</t>
         </is>
       </c>
       <c r="E11" s="15" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>MITIGATED (403 / Off)</t>
         </is>
       </c>
       <c r="F11" s="15" t="inlineStr">
         <is>
-          <t>php-fpm8.1.cve115560_proper</t>
+          <t>C-Binary + SAPI + Edge</t>
         </is>
       </c>
       <c r="G11" s="16" t="inlineStr">
         <is>
-          <t>Pristine binary -&gt; key-sanitized C-binary built &amp; running</t>
+          <t>php-fpm8.1.cve115560_proper (C key sanitizer) · edge 403</t>
         </is>
       </c>
     </row>
@@ -1712,27 +1732,27 @@
       </c>
       <c r="C12" s="12" t="inlineStr">
         <is>
-          <t>VULNERABLE (200)</t>
+          <t>Container Hardening</t>
         </is>
       </c>
       <c r="D12" s="12" t="inlineStr">
         <is>
-          <t>MITIGATED (403/Off)</t>
+          <t>UNHARDENED (SAPI On)</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>HARDENED (SAPI Off)</t>
         </is>
       </c>
       <c r="F12" s="12" t="inlineStr">
         <is>
-          <t>cve-115560-ini-dropin</t>
+          <t>SAPI INI Drop-in</t>
         </is>
       </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
-          <t>Docker container runtime verified Off</t>
+          <t>test-cross-os-e2e.sh debian12 · SAPI verified Off</t>
         </is>
       </c>
     </row>
@@ -1749,27 +1769,27 @@
       </c>
       <c r="C13" s="15" t="inlineStr">
         <is>
-          <t>VULNERABLE (200)</t>
+          <t>Container Hardening</t>
         </is>
       </c>
       <c r="D13" s="15" t="inlineStr">
         <is>
-          <t>MITIGATED (403/Off)</t>
+          <t>UNHARDENED (SAPI On)</t>
         </is>
       </c>
       <c r="E13" s="15" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>HARDENED (SAPI Off)</t>
         </is>
       </c>
       <c r="F13" s="15" t="inlineStr">
         <is>
-          <t>cve-115560-ini-dropin</t>
+          <t>SAPI INI Drop-in</t>
         </is>
       </c>
       <c r="G13" s="16" t="inlineStr">
         <is>
-          <t>Docker container runtime verified Off</t>
+          <t>test-cross-os-e2e.sh alpine · SAPI verified Off</t>
         </is>
       </c>
     </row>
@@ -1786,27 +1806,27 @@
       </c>
       <c r="C14" s="12" t="inlineStr">
         <is>
-          <t>VULNERABLE (200)</t>
+          <t>Container Hardening</t>
         </is>
       </c>
       <c r="D14" s="12" t="inlineStr">
         <is>
-          <t>MITIGATED (403/Off)</t>
+          <t>UNHARDENED (SAPI On)</t>
         </is>
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>HARDENED (SAPI Off)</t>
         </is>
       </c>
       <c r="F14" s="12" t="inlineStr">
         <is>
-          <t>cve-115560-ini-dropin</t>
+          <t>SAPI INI Drop-in</t>
         </is>
       </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
-          <t>Docker live FPM daemon runtime verified Off</t>
+          <t>test-cross-os-e2e.sh php84 · live FPM SAPI Off</t>
         </is>
       </c>
     </row>
@@ -2488,13 +2508,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="62" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2538,6 +2559,11 @@
           <t>Discriminator / Evidence</t>
         </is>
       </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
@@ -2555,9 +2581,14 @@
           <t>HTTP 403 Forbidden</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>Nginx snippet drops PHP_SESSION_UPLOAD_PROGRESS marker at edge</t>
+        </is>
+      </c>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -2577,9 +2608,14 @@
           <t>HTTP 400 / 403</t>
         </is>
       </c>
-      <c r="D7" s="16" t="inlineStr">
+      <c r="D7" s="15" t="inlineStr">
         <is>
           <t>CRLF boundary tampering rejected before FastCGI execution</t>
+        </is>
+      </c>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -2599,9 +2635,14 @@
           <t>enabled =&gt; Off</t>
         </is>
       </c>
-      <c r="D8" s="14" t="inlineStr">
+      <c r="D8" s="12" t="inlineStr">
         <is>
           <t>SAPI drop-in disables upload progress tracking globally</t>
+        </is>
+      </c>
+      <c r="E8" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -2621,9 +2662,14 @@
           <t>Empty session ([])</t>
         </is>
       </c>
-      <c r="D9" s="16" t="inlineStr">
-        <is>
-          <t>INCONCLUSIVE delta (default PHP serializer returns empty keys)</t>
+      <c r="D9" s="15" t="inlineStr">
+        <is>
+          <t>Stock binary also returns empty keys without custom handler</t>
+        </is>
+      </c>
+      <c r="E9" s="19" t="inlineStr">
+        <is>
+          <t>INCONCLUSIVE</t>
         </is>
       </c>
     </row>
@@ -2643,9 +2689,14 @@
           <t>Progress registered</t>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr">
-        <is>
-          <t>PASS — legitimate upload progress functionality preserved</t>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>Legitimate upload progress functionality preserved</t>
+        </is>
+      </c>
+      <c r="E10" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -2665,9 +2716,14 @@
           <t>Both patches applied</t>
         </is>
       </c>
-      <c r="D11" s="16" t="inlineStr">
+      <c r="D11" s="15" t="inlineStr">
         <is>
           <t>Clean textual application (--fuzz=0, exit 0) on shared tree</t>
+        </is>
+      </c>
+      <c r="E11" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -2687,17 +2743,22 @@
           <t>HTTP 200 OK</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>PASS — regular HTTP traffic completely unaffected</t>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>Regular HTTP traffic completely unaffected</t>
+        </is>
+      </c>
+      <c r="E12" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:D12"/>
+  <autoFilter ref="A5:E12"/>
   <mergeCells count="2">
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A3:E3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2848,7 +2909,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>Each target verifies: --preview, --apply, drop-in contents, live FPM SAPI Off, and --rollback.</t>
         </is>

</xml_diff>